<commit_message>
Add LBO / IRR tab with toggles, debt schedule and scenario sensitivity
New 'LBO' sheet built off the FY2021-FY2025 financials:
- Toggle inputs for cash, debt (leverage), interest, fees, mandatory
  amortization, cash sweep and entry/exit multiples (gold cells)
- Base/Bull/Bear scenario selector driving revenue growth, EBITDA margin
  and capex, with defaults anchored to FY21-25 history
- Sources & uses (balances to zero)
- 5-year owner-earnings projection with a beginning-debt interest schedule
  (no circularity), cash sweep and net-debt walk
- Exit returns: MOIC and IRR (closed-form plus a live =IRR on equity CFs)
- Entry x exit EV/EBITDA IRR and MOIC sensitivity grids

Base case returns ~2.6x / ~21% IRR; verified sources=uses and IRR/MOIC
against an independent Python replication.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013eZCyt7rNS6obQfexTe76K
</commit_message>
<xml_diff>
--- a/models/RY_Tool_3_Statement_Model.xlsx
+++ b/models/RY_Tool_3_Statement_Model.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Model" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LBO" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="167" formatCode="0.00&quot;x&quot;;(0.00&quot;x&quot;);\-"/>
     <numFmt numFmtId="168" formatCode="0&quot; days&quot;;(0);\-"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,8 +92,48 @@
       <color rgb="FF404040"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +153,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFCAD2C5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,6 +256,113 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5199,4 +5352,2016 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:L108"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="1.4" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="12.5" customWidth="1" min="3" max="3"/>
+    <col width="12.5" customWidth="1" min="4" max="4"/>
+    <col width="12.5" customWidth="1" min="5" max="5"/>
+    <col width="12.5" customWidth="1" min="6" max="6"/>
+    <col width="12.5" customWidth="1" min="7" max="7"/>
+    <col width="12.5" customWidth="1" min="8" max="8"/>
+    <col width="12.5" customWidth="1" min="9" max="9"/>
+    <col width="12.5" customWidth="1" min="10" max="10"/>
+    <col width="12.5" customWidth="1" min="11" max="11"/>
+    <col width="12.5" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>R. &amp; Y. Tool and Die Co. Limited — LBO / IRR Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="31" t="inlineStr">
+        <is>
+          <t>Owner-earnings LBO built off the FY2021–FY2025 financials (Model tab). Canadian dollars, whole $. Gold cells are toggles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Interest accrues on beginning-of-year debt (no circularity). Excess free cash sweeps to debt paydown; no interim distributions, so equity is entry-in / exit-out. Base-case operating assumptions default to FY21–25 history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>SCENARIO  (Base / Bull / Bear):</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>SCENARIO INPUTS</t>
+        </is>
+      </c>
+      <c r="J5" s="35" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="K5" s="35" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="L5" s="35" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="H6" s="36" t="inlineStr">
+        <is>
+          <t>Revenue growth (%/yr)</t>
+        </is>
+      </c>
+      <c r="J6" s="37" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K6" s="37" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L6" s="37" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>ENTRY, FINANCING &amp; OPERATING ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>EBITDA margin (%)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="39" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="K7" s="39" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="L7" s="39" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="n"/>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Entry (base year = FY2025)</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="n"/>
+      <c r="D8" s="40" t="n"/>
+      <c r="E8" s="40" t="n"/>
+      <c r="F8" s="40" t="n"/>
+      <c r="G8" s="40" t="n"/>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>Capex (% of revenue)</t>
+        </is>
+      </c>
+      <c r="I8" s="40" t="n"/>
+      <c r="J8" s="42" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K8" s="42" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L8" s="42" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="36" t="inlineStr">
+        <is>
+          <t>Entry LTM EBITDA (FY2025)</t>
+        </is>
+      </c>
+      <c r="C9" s="43">
+        <f>'Model'!G45</f>
+        <v/>
+      </c>
+      <c r="D9" s="44" t="inlineStr">
+        <is>
+          <t>Linked from Model — EBITDA bridge.</t>
+        </is>
+      </c>
+      <c r="H9" s="45" t="inlineStr">
+        <is>
+          <t>Historical FY21–25 anchor:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="36" t="inlineStr">
+        <is>
+          <t>Entry LTM revenue (FY2025)</t>
+        </is>
+      </c>
+      <c r="C10" s="43">
+        <f>'Model'!G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="45" t="inlineStr">
+        <is>
+          <t>rev CAGR ~10% · avg EBITDA margin ~17% · avg capex ~3–4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>Entry EV / EBITDA multiple  (x)</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="44" t="inlineStr">
+        <is>
+          <t>Purchase multiple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>Enterprise value at entry</t>
+        </is>
+      </c>
+      <c r="C12" s="43">
+        <f>C9*C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="n"/>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Financing (toggles)</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="n"/>
+      <c r="D13" s="40" t="n"/>
+      <c r="E13" s="40" t="n"/>
+      <c r="F13" s="40" t="n"/>
+      <c r="G13" s="40" t="n"/>
+      <c r="H13" s="40" t="n"/>
+      <c r="I13" s="40" t="n"/>
+      <c r="J13" s="40" t="n"/>
+      <c r="K13" s="40" t="n"/>
+      <c r="L13" s="40" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>Entry leverage — Debt / EBITDA (x)</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D14" s="44" t="inlineStr">
+        <is>
+          <t>DEBT toggle — turns of EBITDA financed with debt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>New debt raised at entry</t>
+        </is>
+      </c>
+      <c r="C15" s="43">
+        <f>C14*C9</f>
+        <v/>
+      </c>
+      <c r="D15" s="44">
+        <f> leverage × entry EBITDA.</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>Interest rate on debt  (%)</t>
+        </is>
+      </c>
+      <c r="C16" s="47" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D16" s="44" t="inlineStr">
+        <is>
+          <t>INTEREST toggle — accrues on opening debt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>Mandatory amortization (% opening debt/yr)</t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>Cash sweep (% of FCF after mandatory)</t>
+        </is>
+      </c>
+      <c r="C18" s="47" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>Minimum / opening cash on balance sheet</t>
+        </is>
+      </c>
+      <c r="C19" s="48" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D19" s="44" t="inlineStr">
+        <is>
+          <t>CASH toggle — cash funded onto the B/S at close and held as a floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="36" t="inlineStr">
+        <is>
+          <t>Transaction &amp; financing fees (% of EV)</t>
+        </is>
+      </c>
+      <c r="C20" s="47" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="n"/>
+      <c r="B21" s="41" t="inlineStr">
+        <is>
+          <t>Operating (scenario-driven; base = FY21–25 history)</t>
+        </is>
+      </c>
+      <c r="C21" s="40" t="n"/>
+      <c r="D21" s="40" t="n"/>
+      <c r="E21" s="40" t="n"/>
+      <c r="F21" s="40" t="n"/>
+      <c r="G21" s="40" t="n"/>
+      <c r="H21" s="40" t="n"/>
+      <c r="I21" s="40" t="n"/>
+      <c r="J21" s="40" t="n"/>
+      <c r="K21" s="40" t="n"/>
+      <c r="L21" s="40" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="36" t="inlineStr">
+        <is>
+          <t>Revenue growth  (%/yr)</t>
+        </is>
+      </c>
+      <c r="C22" s="49">
+        <f>INDEX($J6:$L6,MATCH($C$5,$J$5:$L$5,0))</f>
+        <v/>
+      </c>
+      <c r="D22" s="44" t="inlineStr">
+        <is>
+          <t>Driven by the scenario selector (C5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="36" t="inlineStr">
+        <is>
+          <t>EBITDA margin  (%)</t>
+        </is>
+      </c>
+      <c r="C23" s="49">
+        <f>INDEX($J7:$L7,MATCH($C$5,$J$5:$L$5,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>Capex  (% of revenue)</t>
+        </is>
+      </c>
+      <c r="C24" s="49">
+        <f>INDEX($J8:$L8,MATCH($C$5,$J$5:$L$5,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="36" t="inlineStr">
+        <is>
+          <t>D&amp;A  (% of revenue)</t>
+        </is>
+      </c>
+      <c r="C25" s="47" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D25" s="44" t="inlineStr">
+        <is>
+          <t>Roughly the FY25 run-rate; drives the tax shield.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="36" t="inlineStr">
+        <is>
+          <t>Cash tax rate  (%)</t>
+        </is>
+      </c>
+      <c r="C26" s="47" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D26" s="44" t="inlineStr">
+        <is>
+          <t>≈ FY25 effective rate / CDN small-business rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>Δ Net working capital (% of Δrevenue)</t>
+        </is>
+      </c>
+      <c r="C27" s="47" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="36" t="inlineStr">
+        <is>
+          <t>Exit year  (1–5)</t>
+        </is>
+      </c>
+      <c r="C28" s="50" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>Exit EV / EBITDA multiple  (x)</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" s="44" t="inlineStr">
+        <is>
+          <t>Default = entry multiple (no multiple expansion).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>SOURCES &amp; USES OF FUNDS</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="40" t="n"/>
+      <c r="B32" s="41" t="inlineStr">
+        <is>
+          <t>Uses</t>
+        </is>
+      </c>
+      <c r="C32" s="40" t="n"/>
+      <c r="D32" s="40" t="n"/>
+      <c r="E32" s="40" t="n"/>
+      <c r="F32" s="40" t="n"/>
+      <c r="G32" s="40" t="n"/>
+      <c r="H32" s="40" t="n"/>
+      <c r="I32" s="40" t="n"/>
+      <c r="J32" s="40" t="n"/>
+      <c r="K32" s="40" t="n"/>
+      <c r="L32" s="40" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="36" t="inlineStr">
+        <is>
+          <t>Purchase of enterprise value</t>
+        </is>
+      </c>
+      <c r="C33" s="43">
+        <f>C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="36" t="inlineStr">
+        <is>
+          <t>Cash funded to balance sheet</t>
+        </is>
+      </c>
+      <c r="C34" s="43">
+        <f>C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="36" t="inlineStr">
+        <is>
+          <t>Transaction &amp; financing fees</t>
+        </is>
+      </c>
+      <c r="C35" s="43">
+        <f>C20*C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Total uses</t>
+        </is>
+      </c>
+      <c r="C36" s="51">
+        <f>SUM(C33:C35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="40" t="n"/>
+      <c r="B37" s="41" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="C37" s="40" t="n"/>
+      <c r="D37" s="40" t="n"/>
+      <c r="E37" s="40" t="n"/>
+      <c r="F37" s="40" t="n"/>
+      <c r="G37" s="40" t="n"/>
+      <c r="H37" s="40" t="n"/>
+      <c r="I37" s="40" t="n"/>
+      <c r="J37" s="40" t="n"/>
+      <c r="K37" s="40" t="n"/>
+      <c r="L37" s="40" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>New debt raised</t>
+        </is>
+      </c>
+      <c r="C38" s="43">
+        <f>C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>Sponsor equity (plug)</t>
+        </is>
+      </c>
+      <c r="C39" s="52">
+        <f>C36-C38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="32" t="inlineStr">
+        <is>
+          <t>Total sources</t>
+        </is>
+      </c>
+      <c r="C40" s="51">
+        <f>C38+C39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="36" t="inlineStr">
+        <is>
+          <t>Check (sources − uses)</t>
+        </is>
+      </c>
+      <c r="C41" s="43">
+        <f>C40-C36</f>
+        <v/>
+      </c>
+      <c r="D41" s="44" t="inlineStr">
+        <is>
+          <t>Must be 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="36" t="inlineStr">
+        <is>
+          <t>Entry net debt (debt − opening cash)</t>
+        </is>
+      </c>
+      <c r="C42" s="43">
+        <f>C38-C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="38" t="inlineStr">
+        <is>
+          <t>OWNER-EARNINGS PROJECTION, DEBT SCHEDULE &amp; FREE CASH FLOW</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="53" t="n"/>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>($)</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>FY2025  (entry)</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="54" t="inlineStr">
+        <is>
+          <t>Hold year (0 = entry)</t>
+        </is>
+      </c>
+      <c r="G47" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="J47" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="L47" s="55" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C48" s="52">
+        <f>'Model'!C9</f>
+        <v/>
+      </c>
+      <c r="D48" s="52">
+        <f>'Model'!D9</f>
+        <v/>
+      </c>
+      <c r="E48" s="52">
+        <f>'Model'!E9</f>
+        <v/>
+      </c>
+      <c r="F48" s="52">
+        <f>'Model'!F9</f>
+        <v/>
+      </c>
+      <c r="G48" s="52">
+        <f>'Model'!G9</f>
+        <v/>
+      </c>
+      <c r="H48" s="52">
+        <f>G48*(1+$C$22)</f>
+        <v/>
+      </c>
+      <c r="I48" s="52">
+        <f>H48*(1+$C$22)</f>
+        <v/>
+      </c>
+      <c r="J48" s="52">
+        <f>I48*(1+$C$22)</f>
+        <v/>
+      </c>
+      <c r="K48" s="52">
+        <f>J48*(1+$C$22)</f>
+        <v/>
+      </c>
+      <c r="L48" s="52">
+        <f>K48*(1+$C$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Revenue growth %</t>
+        </is>
+      </c>
+      <c r="D49" s="56">
+        <f>IFERROR(D48/C48-1,"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="56">
+        <f>IFERROR(E48/D48-1,"")</f>
+        <v/>
+      </c>
+      <c r="F49" s="56">
+        <f>IFERROR(F48/E48-1,"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="56">
+        <f>IFERROR(G48/F48-1,"")</f>
+        <v/>
+      </c>
+      <c r="H49" s="56">
+        <f>IFERROR(H48/G48-1,"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="56">
+        <f>IFERROR(I48/H48-1,"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="56">
+        <f>IFERROR(J48/I48-1,"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="56">
+        <f>IFERROR(K48/J48-1,"")</f>
+        <v/>
+      </c>
+      <c r="L49" s="56">
+        <f>IFERROR(L48/K48-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="32" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="C50" s="51">
+        <f>'Model'!C45</f>
+        <v/>
+      </c>
+      <c r="D50" s="51">
+        <f>'Model'!D45</f>
+        <v/>
+      </c>
+      <c r="E50" s="51">
+        <f>'Model'!E45</f>
+        <v/>
+      </c>
+      <c r="F50" s="51">
+        <f>'Model'!F45</f>
+        <v/>
+      </c>
+      <c r="G50" s="51">
+        <f>'Model'!G45</f>
+        <v/>
+      </c>
+      <c r="H50" s="51">
+        <f>H48*$C$23</f>
+        <v/>
+      </c>
+      <c r="I50" s="51">
+        <f>I48*$C$23</f>
+        <v/>
+      </c>
+      <c r="J50" s="51">
+        <f>J48*$C$23</f>
+        <v/>
+      </c>
+      <c r="K50" s="51">
+        <f>K48*$C$23</f>
+        <v/>
+      </c>
+      <c r="L50" s="51">
+        <f>L48*$C$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EBITDA margin %</t>
+        </is>
+      </c>
+      <c r="C51" s="56">
+        <f>IFERROR(C50/C48,"")</f>
+        <v/>
+      </c>
+      <c r="D51" s="56">
+        <f>IFERROR(D50/D48,"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="56">
+        <f>IFERROR(E50/E48,"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="56">
+        <f>IFERROR(F50/F48,"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="56">
+        <f>IFERROR(G50/G48,"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="56">
+        <f>IFERROR(H50/H48,"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="56">
+        <f>IFERROR(I50/I48,"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="56">
+        <f>IFERROR(J50/J48,"")</f>
+        <v/>
+      </c>
+      <c r="K51" s="56">
+        <f>IFERROR(K50/K48,"")</f>
+        <v/>
+      </c>
+      <c r="L51" s="56">
+        <f>IFERROR(L50/L48,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="36" t="inlineStr">
+        <is>
+          <t>Depreciation &amp; amortization</t>
+        </is>
+      </c>
+      <c r="C52" s="43">
+        <f>'Model'!C151</f>
+        <v/>
+      </c>
+      <c r="D52" s="43">
+        <f>'Model'!D151</f>
+        <v/>
+      </c>
+      <c r="E52" s="43">
+        <f>'Model'!E151</f>
+        <v/>
+      </c>
+      <c r="F52" s="43">
+        <f>'Model'!F151</f>
+        <v/>
+      </c>
+      <c r="G52" s="43">
+        <f>'Model'!G151</f>
+        <v/>
+      </c>
+      <c r="H52" s="43">
+        <f>H48*$C$25</f>
+        <v/>
+      </c>
+      <c r="I52" s="43">
+        <f>I48*$C$25</f>
+        <v/>
+      </c>
+      <c r="J52" s="43">
+        <f>J48*$C$25</f>
+        <v/>
+      </c>
+      <c r="K52" s="43">
+        <f>K48*$C$25</f>
+        <v/>
+      </c>
+      <c r="L52" s="43">
+        <f>L48*$C$25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="32" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="C53" s="51">
+        <f>C50-C52</f>
+        <v/>
+      </c>
+      <c r="D53" s="51">
+        <f>D50-D52</f>
+        <v/>
+      </c>
+      <c r="E53" s="51">
+        <f>E50-E52</f>
+        <v/>
+      </c>
+      <c r="F53" s="51">
+        <f>F50-F52</f>
+        <v/>
+      </c>
+      <c r="G53" s="51">
+        <f>G50-G52</f>
+        <v/>
+      </c>
+      <c r="H53" s="51">
+        <f>H50-H52</f>
+        <v/>
+      </c>
+      <c r="I53" s="51">
+        <f>I50-I52</f>
+        <v/>
+      </c>
+      <c r="J53" s="51">
+        <f>J50-J52</f>
+        <v/>
+      </c>
+      <c r="K53" s="51">
+        <f>K50-K52</f>
+        <v/>
+      </c>
+      <c r="L53" s="51">
+        <f>L50-L52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="36" t="inlineStr">
+        <is>
+          <t>Interest expense (on opening debt)</t>
+        </is>
+      </c>
+      <c r="H54" s="43">
+        <f>$C$16*H64</f>
+        <v/>
+      </c>
+      <c r="I54" s="43">
+        <f>$C$16*I64</f>
+        <v/>
+      </c>
+      <c r="J54" s="43">
+        <f>$C$16*J64</f>
+        <v/>
+      </c>
+      <c r="K54" s="43">
+        <f>$C$16*K64</f>
+        <v/>
+      </c>
+      <c r="L54" s="43">
+        <f>$C$16*L64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="32" t="inlineStr">
+        <is>
+          <t>Pre-tax profit (EBT)</t>
+        </is>
+      </c>
+      <c r="H55" s="51">
+        <f>H53-H54</f>
+        <v/>
+      </c>
+      <c r="I55" s="51">
+        <f>I53-I54</f>
+        <v/>
+      </c>
+      <c r="J55" s="51">
+        <f>J53-J54</f>
+        <v/>
+      </c>
+      <c r="K55" s="51">
+        <f>K53-K54</f>
+        <v/>
+      </c>
+      <c r="L55" s="51">
+        <f>L53-L54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="36" t="inlineStr">
+        <is>
+          <t>Cash taxes</t>
+        </is>
+      </c>
+      <c r="H56" s="43">
+        <f>-MAX(H55*$C$26,0)</f>
+        <v/>
+      </c>
+      <c r="I56" s="43">
+        <f>-MAX(I55*$C$26,0)</f>
+        <v/>
+      </c>
+      <c r="J56" s="43">
+        <f>-MAX(J55*$C$26,0)</f>
+        <v/>
+      </c>
+      <c r="K56" s="43">
+        <f>-MAX(K55*$C$26,0)</f>
+        <v/>
+      </c>
+      <c r="L56" s="43">
+        <f>-MAX(L55*$C$26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="32" t="inlineStr">
+        <is>
+          <t>Net profit after tax</t>
+        </is>
+      </c>
+      <c r="H57" s="51">
+        <f>H55+H56</f>
+        <v/>
+      </c>
+      <c r="I57" s="51">
+        <f>I55+I56</f>
+        <v/>
+      </c>
+      <c r="J57" s="51">
+        <f>J55+J56</f>
+        <v/>
+      </c>
+      <c r="K57" s="51">
+        <f>K55+K56</f>
+        <v/>
+      </c>
+      <c r="L57" s="51">
+        <f>L55+L56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (+) D&amp;A</t>
+        </is>
+      </c>
+      <c r="H58" s="43">
+        <f>H52</f>
+        <v/>
+      </c>
+      <c r="I58" s="43">
+        <f>I52</f>
+        <v/>
+      </c>
+      <c r="J58" s="43">
+        <f>J52</f>
+        <v/>
+      </c>
+      <c r="K58" s="43">
+        <f>K52</f>
+        <v/>
+      </c>
+      <c r="L58" s="43">
+        <f>L52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (−) Capex</t>
+        </is>
+      </c>
+      <c r="H59" s="43">
+        <f>-H48*$C$24</f>
+        <v/>
+      </c>
+      <c r="I59" s="43">
+        <f>-I48*$C$24</f>
+        <v/>
+      </c>
+      <c r="J59" s="43">
+        <f>-J48*$C$24</f>
+        <v/>
+      </c>
+      <c r="K59" s="43">
+        <f>-K48*$C$24</f>
+        <v/>
+      </c>
+      <c r="L59" s="43">
+        <f>-L48*$C$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (−) Δ Net working capital</t>
+        </is>
+      </c>
+      <c r="H60" s="43">
+        <f>-(H48-G48)*$C$27</f>
+        <v/>
+      </c>
+      <c r="I60" s="43">
+        <f>-(I48-H48)*$C$27</f>
+        <v/>
+      </c>
+      <c r="J60" s="43">
+        <f>-(J48-I48)*$C$27</f>
+        <v/>
+      </c>
+      <c r="K60" s="43">
+        <f>-(K48-J48)*$C$27</f>
+        <v/>
+      </c>
+      <c r="L60" s="43">
+        <f>-(L48-K48)*$C$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>Levered free cash flow (owner earnings)</t>
+        </is>
+      </c>
+      <c r="H61" s="51">
+        <f>H57+H58+H59+H60</f>
+        <v/>
+      </c>
+      <c r="I61" s="51">
+        <f>I57+I58+I59+I60</f>
+        <v/>
+      </c>
+      <c r="J61" s="51">
+        <f>J57+J58+J59+J60</f>
+        <v/>
+      </c>
+      <c r="K61" s="51">
+        <f>K57+K58+K59+K60</f>
+        <v/>
+      </c>
+      <c r="L61" s="51">
+        <f>L57+L58+L59+L60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="40" t="n"/>
+      <c r="B63" s="41" t="inlineStr">
+        <is>
+          <t>Debt schedule</t>
+        </is>
+      </c>
+      <c r="C63" s="40" t="n"/>
+      <c r="D63" s="40" t="n"/>
+      <c r="E63" s="40" t="n"/>
+      <c r="F63" s="40" t="n"/>
+      <c r="G63" s="40" t="n"/>
+      <c r="H63" s="40" t="n"/>
+      <c r="I63" s="40" t="n"/>
+      <c r="J63" s="40" t="n"/>
+      <c r="K63" s="40" t="n"/>
+      <c r="L63" s="40" t="n"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="36" t="inlineStr">
+        <is>
+          <t>Beginning debt</t>
+        </is>
+      </c>
+      <c r="H64" s="43">
+        <f>G67</f>
+        <v/>
+      </c>
+      <c r="I64" s="43">
+        <f>H67</f>
+        <v/>
+      </c>
+      <c r="J64" s="43">
+        <f>I67</f>
+        <v/>
+      </c>
+      <c r="K64" s="43">
+        <f>J67</f>
+        <v/>
+      </c>
+      <c r="L64" s="43">
+        <f>K67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (−) Mandatory amortization</t>
+        </is>
+      </c>
+      <c r="H65" s="43">
+        <f>-MIN(H64,$C$17*$C$15)</f>
+        <v/>
+      </c>
+      <c r="I65" s="43">
+        <f>-MIN(I64,$C$17*$C$15)</f>
+        <v/>
+      </c>
+      <c r="J65" s="43">
+        <f>-MIN(J64,$C$17*$C$15)</f>
+        <v/>
+      </c>
+      <c r="K65" s="43">
+        <f>-MIN(K64,$C$17*$C$15)</f>
+        <v/>
+      </c>
+      <c r="L65" s="43">
+        <f>-MIN(L64,$C$17*$C$15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (−) Cash sweep</t>
+        </is>
+      </c>
+      <c r="H66" s="43">
+        <f>-MIN(MAX(H61+H65,0)*$C$18,H64+H65)</f>
+        <v/>
+      </c>
+      <c r="I66" s="43">
+        <f>-MIN(MAX(I61+I65,0)*$C$18,I64+I65)</f>
+        <v/>
+      </c>
+      <c r="J66" s="43">
+        <f>-MIN(MAX(J61+J65,0)*$C$18,J64+J65)</f>
+        <v/>
+      </c>
+      <c r="K66" s="43">
+        <f>-MIN(MAX(K61+K65,0)*$C$18,K64+K65)</f>
+        <v/>
+      </c>
+      <c r="L66" s="43">
+        <f>-MIN(MAX(L61+L65,0)*$C$18,L64+L65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="32" t="inlineStr">
+        <is>
+          <t>Ending debt</t>
+        </is>
+      </c>
+      <c r="G67" s="43">
+        <f>$C$15</f>
+        <v/>
+      </c>
+      <c r="H67" s="51">
+        <f>H64+H65+H66</f>
+        <v/>
+      </c>
+      <c r="I67" s="51">
+        <f>I64+I65+I66</f>
+        <v/>
+      </c>
+      <c r="J67" s="51">
+        <f>J64+J65+J66</f>
+        <v/>
+      </c>
+      <c r="K67" s="51">
+        <f>K64+K65+K66</f>
+        <v/>
+      </c>
+      <c r="L67" s="51">
+        <f>L64+L65+L66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="40" t="n"/>
+      <c r="B69" s="41" t="inlineStr">
+        <is>
+          <t>Cash &amp; leverage</t>
+        </is>
+      </c>
+      <c r="C69" s="40" t="n"/>
+      <c r="D69" s="40" t="n"/>
+      <c r="E69" s="40" t="n"/>
+      <c r="F69" s="40" t="n"/>
+      <c r="G69" s="40" t="n"/>
+      <c r="H69" s="40" t="n"/>
+      <c r="I69" s="40" t="n"/>
+      <c r="J69" s="40" t="n"/>
+      <c r="K69" s="40" t="n"/>
+      <c r="L69" s="40" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="36" t="inlineStr">
+        <is>
+          <t>Beginning cash</t>
+        </is>
+      </c>
+      <c r="H70" s="43">
+        <f>G72</f>
+        <v/>
+      </c>
+      <c r="I70" s="43">
+        <f>H72</f>
+        <v/>
+      </c>
+      <c r="J70" s="43">
+        <f>I72</f>
+        <v/>
+      </c>
+      <c r="K70" s="43">
+        <f>J72</f>
+        <v/>
+      </c>
+      <c r="L70" s="43">
+        <f>K72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (+) FCF after debt paydown</t>
+        </is>
+      </c>
+      <c r="H71" s="43">
+        <f>H61+H65+H66</f>
+        <v/>
+      </c>
+      <c r="I71" s="43">
+        <f>I61+I65+I66</f>
+        <v/>
+      </c>
+      <c r="J71" s="43">
+        <f>J61+J65+J66</f>
+        <v/>
+      </c>
+      <c r="K71" s="43">
+        <f>K61+K65+K66</f>
+        <v/>
+      </c>
+      <c r="L71" s="43">
+        <f>L61+L65+L66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="32" t="inlineStr">
+        <is>
+          <t>Ending cash</t>
+        </is>
+      </c>
+      <c r="G72" s="43">
+        <f>$C$19</f>
+        <v/>
+      </c>
+      <c r="H72" s="51">
+        <f>H70+H71</f>
+        <v/>
+      </c>
+      <c r="I72" s="51">
+        <f>I70+I71</f>
+        <v/>
+      </c>
+      <c r="J72" s="51">
+        <f>J70+J71</f>
+        <v/>
+      </c>
+      <c r="K72" s="51">
+        <f>K70+K71</f>
+        <v/>
+      </c>
+      <c r="L72" s="51">
+        <f>L70+L71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="36" t="inlineStr">
+        <is>
+          <t>Net debt (debt − cash)</t>
+        </is>
+      </c>
+      <c r="G73" s="43">
+        <f>G67-G72</f>
+        <v/>
+      </c>
+      <c r="H73" s="43">
+        <f>H67-H72</f>
+        <v/>
+      </c>
+      <c r="I73" s="43">
+        <f>I67-I72</f>
+        <v/>
+      </c>
+      <c r="J73" s="43">
+        <f>J67-J72</f>
+        <v/>
+      </c>
+      <c r="K73" s="43">
+        <f>K67-K72</f>
+        <v/>
+      </c>
+      <c r="L73" s="43">
+        <f>L67-L72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net debt / EBITDA  (x)</t>
+        </is>
+      </c>
+      <c r="G74" s="57">
+        <f>IFERROR(G73/G50,"")</f>
+        <v/>
+      </c>
+      <c r="H74" s="57">
+        <f>IFERROR(H73/H50,"")</f>
+        <v/>
+      </c>
+      <c r="I74" s="57">
+        <f>IFERROR(I73/I50,"")</f>
+        <v/>
+      </c>
+      <c r="J74" s="57">
+        <f>IFERROR(J73/J50,"")</f>
+        <v/>
+      </c>
+      <c r="K74" s="57">
+        <f>IFERROR(K73/K50,"")</f>
+        <v/>
+      </c>
+      <c r="L74" s="57">
+        <f>IFERROR(L73/L50,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n"/>
+      <c r="B76" s="38" t="inlineStr">
+        <is>
+          <t>RETURNS — EXIT &amp; IRR</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="n"/>
+      <c r="D76" s="4" t="n"/>
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
+      <c r="J76" s="4" t="n"/>
+      <c r="K76" s="4" t="n"/>
+      <c r="L76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="36" t="inlineStr">
+        <is>
+          <t>Hold period (years)</t>
+        </is>
+      </c>
+      <c r="C77" s="58">
+        <f>C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="36" t="inlineStr">
+        <is>
+          <t>Exit-year EBITDA</t>
+        </is>
+      </c>
+      <c r="C78" s="43">
+        <f>INDEX($G50:$L50,1,$C$28+1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="36" t="inlineStr">
+        <is>
+          <t>Exit EV / EBITDA multiple  (x)</t>
+        </is>
+      </c>
+      <c r="C79" s="59">
+        <f>C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="36" t="inlineStr">
+        <is>
+          <t>Exit enterprise value</t>
+        </is>
+      </c>
+      <c r="C80" s="43">
+        <f>C78*C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="36" t="inlineStr">
+        <is>
+          <t>(−) Net debt at exit</t>
+        </is>
+      </c>
+      <c r="C81" s="43">
+        <f>INDEX($G73:$L73,1,$C$28+1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="32" t="inlineStr">
+        <is>
+          <t>Exit equity value</t>
+        </is>
+      </c>
+      <c r="C82" s="51">
+        <f>C80-C81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="36" t="inlineStr">
+        <is>
+          <t>Entry sponsor equity</t>
+        </is>
+      </c>
+      <c r="C83" s="43">
+        <f>C39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="32" t="inlineStr">
+        <is>
+          <t>MOIC  (x)</t>
+        </is>
+      </c>
+      <c r="C84" s="60">
+        <f>IFERROR(C82/C83,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="32" t="inlineStr">
+        <is>
+          <t>IRR  (equity, closed form)</t>
+        </is>
+      </c>
+      <c r="C85" s="61">
+        <f>IFERROR((C82/C83)^(1/C77)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="40" t="n"/>
+      <c r="B87" s="41" t="inlineStr">
+        <is>
+          <t>Equity cash flows (Year 0 → exit)   —   live =IRR()</t>
+        </is>
+      </c>
+      <c r="C87" s="40" t="n"/>
+      <c r="D87" s="40" t="n"/>
+      <c r="E87" s="40" t="n"/>
+      <c r="F87" s="40" t="n"/>
+      <c r="G87" s="40" t="n"/>
+      <c r="H87" s="40" t="n"/>
+      <c r="I87" s="40" t="n"/>
+      <c r="J87" s="40" t="n"/>
+      <c r="K87" s="40" t="n"/>
+      <c r="L87" s="40" t="n"/>
+    </row>
+    <row r="88">
+      <c r="B88" s="36" t="inlineStr">
+        <is>
+          <t>Sponsor equity cash flow</t>
+        </is>
+      </c>
+      <c r="G88" s="43">
+        <f>-C39</f>
+        <v/>
+      </c>
+      <c r="H88" s="43">
+        <f>IF($C$28=1,$C$82,0)</f>
+        <v/>
+      </c>
+      <c r="I88" s="43">
+        <f>IF($C$28=2,$C$82,0)</f>
+        <v/>
+      </c>
+      <c r="J88" s="43">
+        <f>IF($C$28=3,$C$82,0)</f>
+        <v/>
+      </c>
+      <c r="K88" s="43">
+        <f>IF($C$28=4,$C$82,0)</f>
+        <v/>
+      </c>
+      <c r="L88" s="43">
+        <f>IF($C$28=5,$C$82,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="32" t="inlineStr">
+        <is>
+          <t>IRR  =IRR(equity cash flows)</t>
+        </is>
+      </c>
+      <c r="C89" s="61">
+        <f>IFERROR(IRR(G88:L88),"")</f>
+        <v/>
+      </c>
+      <c r="D89" s="62" t="inlineStr">
+        <is>
+          <t>Matches the closed-form IRR above; add interim dividends to G88:L88 to extend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n"/>
+      <c r="B92" s="38" t="inlineStr">
+        <is>
+          <t>IRR SENSITIVITY — ENTRY (down) × EXIT (across) EV/EBITDA MULTIPLE</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="n"/>
+      <c r="D92" s="4" t="n"/>
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="n"/>
+      <c r="K92" s="4" t="n"/>
+      <c r="L92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="62" t="inlineStr">
+        <is>
+          <t>Holds the current operating scenario, leverage, interest and cash fixed; only the multiples vary. Live case is highlighted by your C11 / C29 inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="C94" s="63" t="inlineStr">
+        <is>
+          <t>Entry ↓ / Exit →</t>
+        </is>
+      </c>
+      <c r="D94" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="E94" s="64" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F94" s="64" t="n">
+        <v>6</v>
+      </c>
+      <c r="G94" s="64" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H94" s="64" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="C95" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D95" s="65">
+        <f>IFERROR(((D$94*$C$78-$C$81)/($C95*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="E95" s="65">
+        <f>IFERROR(((E$94*$C$78-$C$81)/($C95*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="F95" s="65">
+        <f>IFERROR(((F$94*$C$78-$C$81)/($C95*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="G95" s="65">
+        <f>IFERROR(((G$94*$C$78-$C$81)/($C95*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="H95" s="65">
+        <f>IFERROR(((H$94*$C$78-$C$81)/($C95*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="C96" s="64" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D96" s="65">
+        <f>IFERROR(((D$94*$C$78-$C$81)/($C96*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="E96" s="65">
+        <f>IFERROR(((E$94*$C$78-$C$81)/($C96*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="F96" s="65">
+        <f>IFERROR(((F$94*$C$78-$C$81)/($C96*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="G96" s="65">
+        <f>IFERROR(((G$94*$C$78-$C$81)/($C96*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="H96" s="65">
+        <f>IFERROR(((H$94*$C$78-$C$81)/($C96*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="C97" s="64" t="n">
+        <v>6</v>
+      </c>
+      <c r="D97" s="65">
+        <f>IFERROR(((D$94*$C$78-$C$81)/($C97*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="E97" s="65">
+        <f>IFERROR(((E$94*$C$78-$C$81)/($C97*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="F97" s="65">
+        <f>IFERROR(((F$94*$C$78-$C$81)/($C97*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="G97" s="65">
+        <f>IFERROR(((G$94*$C$78-$C$81)/($C97*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="H97" s="65">
+        <f>IFERROR(((H$94*$C$78-$C$81)/($C97*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="C98" s="64" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D98" s="65">
+        <f>IFERROR(((D$94*$C$78-$C$81)/($C98*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="E98" s="65">
+        <f>IFERROR(((E$94*$C$78-$C$81)/($C98*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="F98" s="65">
+        <f>IFERROR(((F$94*$C$78-$C$81)/($C98*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="G98" s="65">
+        <f>IFERROR(((G$94*$C$78-$C$81)/($C98*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="H98" s="65">
+        <f>IFERROR(((H$94*$C$78-$C$81)/($C98*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="C99" s="64" t="n">
+        <v>7</v>
+      </c>
+      <c r="D99" s="65">
+        <f>IFERROR(((D$94*$C$78-$C$81)/($C99*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="E99" s="65">
+        <f>IFERROR(((E$94*$C$78-$C$81)/($C99*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="F99" s="65">
+        <f>IFERROR(((F$94*$C$78-$C$81)/($C99*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="G99" s="65">
+        <f>IFERROR(((G$94*$C$78-$C$81)/($C99*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+      <c r="H99" s="65">
+        <f>IFERROR(((H$94*$C$78-$C$81)/($C99*$C$9*(1+$C$20)+$C$19-$C$15))^(1/$C$28)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="n"/>
+      <c r="B102" s="38" t="inlineStr">
+        <is>
+          <t>MOIC SENSITIVITY — ENTRY (down) × EXIT (across) EV/EBITDA MULTIPLE</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="n"/>
+      <c r="D102" s="4" t="n"/>
+      <c r="E102" s="4" t="n"/>
+      <c r="F102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
+      <c r="I102" s="4" t="n"/>
+      <c r="J102" s="4" t="n"/>
+      <c r="K102" s="4" t="n"/>
+      <c r="L102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="C103" s="63" t="inlineStr">
+        <is>
+          <t>Entry ↓ / Exit →</t>
+        </is>
+      </c>
+      <c r="D103" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="E103" s="64" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F103" s="64" t="n">
+        <v>6</v>
+      </c>
+      <c r="G103" s="64" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H103" s="64" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="C104" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D104" s="66">
+        <f>IFERROR((D$103*$C$78-$C$81)/($C104*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="E104" s="66">
+        <f>IFERROR((E$103*$C$78-$C$81)/($C104*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="F104" s="66">
+        <f>IFERROR((F$103*$C$78-$C$81)/($C104*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="G104" s="66">
+        <f>IFERROR((G$103*$C$78-$C$81)/($C104*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="H104" s="66">
+        <f>IFERROR((H$103*$C$78-$C$81)/($C104*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="C105" s="64" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D105" s="66">
+        <f>IFERROR((D$103*$C$78-$C$81)/($C105*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="E105" s="66">
+        <f>IFERROR((E$103*$C$78-$C$81)/($C105*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="F105" s="66">
+        <f>IFERROR((F$103*$C$78-$C$81)/($C105*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="G105" s="66">
+        <f>IFERROR((G$103*$C$78-$C$81)/($C105*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="H105" s="66">
+        <f>IFERROR((H$103*$C$78-$C$81)/($C105*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="C106" s="64" t="n">
+        <v>6</v>
+      </c>
+      <c r="D106" s="66">
+        <f>IFERROR((D$103*$C$78-$C$81)/($C106*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="E106" s="66">
+        <f>IFERROR((E$103*$C$78-$C$81)/($C106*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="F106" s="66">
+        <f>IFERROR((F$103*$C$78-$C$81)/($C106*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="G106" s="66">
+        <f>IFERROR((G$103*$C$78-$C$81)/($C106*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="H106" s="66">
+        <f>IFERROR((H$103*$C$78-$C$81)/($C106*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="C107" s="64" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D107" s="66">
+        <f>IFERROR((D$103*$C$78-$C$81)/($C107*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="E107" s="66">
+        <f>IFERROR((E$103*$C$78-$C$81)/($C107*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="F107" s="66">
+        <f>IFERROR((F$103*$C$78-$C$81)/($C107*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="G107" s="66">
+        <f>IFERROR((G$103*$C$78-$C$81)/($C107*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="H107" s="66">
+        <f>IFERROR((H$103*$C$78-$C$81)/($C107*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="C108" s="64" t="n">
+        <v>7</v>
+      </c>
+      <c r="D108" s="66">
+        <f>IFERROR((D$103*$C$78-$C$81)/($C108*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="E108" s="66">
+        <f>IFERROR((E$103*$C$78-$C$81)/($C108*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="F108" s="66">
+        <f>IFERROR((F$103*$C$78-$C$81)/($C108*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="G108" s="66">
+        <f>IFERROR((G$103*$C$78-$C$81)/($C108*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+      <c r="H108" s="66">
+        <f>IFERROR((H$103*$C$78-$C$81)/($C108*$C$9*(1+$C$20)+$C$19-$C$15),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>